<commit_message>
docs(catalog): add Sheet 6 Universal Ticker & Market Coverage to Excel catalog
</commit_message>
<xml_diff>
--- a/agents_and_skills_catalog.xlsx
+++ b/agents_and_skills_catalog.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills Catalog" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NVIDIA Suite" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration Architecture" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ticker &amp; Market Coverage" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -57,7 +58,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +95,12 @@
         <bgColor rgb="004A235A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B365D"/>
+        <bgColor rgb="001B365D"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -121,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -148,6 +155,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -518,10 +528,10 @@
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -664,14 +674,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1302,10 +1312,10 @@
     <col width="43" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1991,9 +2001,9 @@
     <col width="33" customWidth="1" min="1" max="1"/>
     <col width="43" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2272,9 +2282,9 @@
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
     <col width="47" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2550,4 +2560,485 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Market / Asset Class</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Exchange / Region</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>Ticker Suffix &amp; Format</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>Data Pipeline &amp; SEC Engine</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>Supported Capabilities</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>Example Tickers You Can Run</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>How to Access / Run Command</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>US Public Equities (Large, Mid, Small Cap)</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>NYSE, NASDAQ, AMEX (United States)</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Bare symbol: &lt;TICKER&gt; (e.g. AAPL, NVDA, TSLA)</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>SEC EDGAR XBRL (tools/filing.py CIKResolver) + yFinance + DataLayer</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Full primary audited 10-K / 10-Q statement extraction, analytical DCF valuation, capital returns yield, footnote concentration (&gt;10%), verifier re-fetch</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>AAPL, NVDA, MSFT, TSLA, AMZN, GOOGL, META, AMD, LLY, JPM, PLTR, BRK-B, COST, WMT, NFLX, DIS</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>CLI: python run_research.py TSLA 1
+UI: Type TSLA in Streamlit
+Watchlist: Add TSLA to watchlist.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Foreign Private Issuers (ADRs / US Listed)</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>NYSE / NASDAQ (International filers with SEC)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>US listing symbol: &lt;TICKER&gt; (e.g. TSM, ASML, NVO)</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>SEC Form 20-F Parser (tools/filing.py) under ifrs-full taxonomy</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Audited IFRS balance sheet, income statement, operating cash flows, Capex, analytical DCF in USD, SEC CIK resolution</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>TSM (Taiwan Semi), ASML (Netherlands), NVO (Novo Nordisk), BABA (Alibaba), SAP (Germany), AZN (AstraZeneca), SONY (Japan)</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>CLI: python run_research.py TSM 1
+UI: Type TSM in Streamlit
+API: dl.get_fundamentals('TSM')</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Indian Equities (National Stock Exchange)</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>NSE (India)</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Ticker with .NS suffix: &lt;SYMBOL&gt;.NS</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Multi-source DataLayer + Yahoo Finance India + ESEF / Corporate Filing Engine</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Real-time and historical quotes in INR, consolidated P&amp;L, balance sheet, cash flows, DCF valuation with INR currency handling</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>TCS.NS, INFY.NS, RELIANCE.NS, HDFCBANK.NS, TATAMOTORS.NS, ICICIBANK.NS, BHARTIARTL.NS, WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>CLI: python run_research.py TCS.NS 1
+UI: Type TCS.NS in Streamlit
+R: fetch_sec_financials('TCS.NS')</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Indian Equities (Bombay Stock Exchange)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>BSE (India)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Ticker / Scrip code with .BO suffix: &lt;SYMBOL&gt;.BO</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Multi-source DataLayer + yFinance + BSE feeds</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Quotes in INR, multi-source fallback, historical returns, backtesting and screening</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>500325.BO (Reliance), 532540.BO (TCS), 500180.BO (HDFC Bank), 500209.BO (Infosys)</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>CLI: python run_research.py 500325.BO 1
+Watchlist: Add to watchlist.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom Equities</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>London Stock Exchange (LSE, United Kingdom)</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Ticker with .L suffix: &lt;SYMBOL&gt;.L</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Multi-source DataLayer (yFinance + Finnhub) with GBP currency normalization</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Quotes in GBP/GBp, multi-currency conversion via tools/calc/fx.py, historical returns, DCF valuation</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>SHEL.L (Shell), BP.L (BP), HSBA.L (HSBC), AZN.L (AstraZeneca), ULVR.L (Unilever), RIO.L (Rio Tinto)</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>CLI: python run_research.py SHEL.L 1
+R: calc_dcf(...) with currency='GBP'</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>German &amp; European Equities</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>XETRA / Frankfurt (Germany)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Ticker with .DE suffix: &lt;SYMBOL&gt;.DE</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Multi-source DataLayer with EUR currency normalization</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Quotes in EUR, European corporate disclosures, DCF valuation, multi-asset backtesting</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>BMW.DE (BMW), VOW3.DE (Volkswagen), SIE.DE (Siemens), SAP.DE (SAP), ALV.DE (Allianz)</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>CLI: python run_research.py BMW.DE 1
+Quant: BacktestSandbox(['BMW.DE', 'SIE.DE'])</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>French &amp; Euronext Equities</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Euronext Paris (France)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Ticker with .PA suffix: &lt;SYMBOL&gt;.PA</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Multi-source DataLayer with EUR currency normalization</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Quotes in EUR, luxury/industrial fundamentals, cash flow modeling, alert monitoring</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>MC.PA (LVMH), OR.PA (L'Oréal), AIR.PA (Airbus), RMS.PA (Hermès), TTE.PA (TotalEnergies)</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>CLI: python run_research.py MC.PA 1
+UI: Type MC.PA in Streamlit</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Canadian Equities</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Toronto Stock Exchange (TSX, Canada)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Ticker with .TO suffix: &lt;SYMBOL&gt;.TO</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Multi-source DataLayer with CAD currency normalization</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Quotes in CAD, banking &amp; energy fundamentals, DCF valuation, factor screening</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>SHOP.TO (Shopify), RY.TO (Royal Bank of Canada), TD.TO (Toronto-Dominion), ENB.TO (Enbridge)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>CLI: python run_research.py SHOP.TO 1
+Watchlist: Add to watchlist.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Japanese Equities</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Tokyo Stock Exchange (TSE, Japan)</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Numeric ticker with .T suffix: &lt;NUM&gt;.T</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Multi-source DataLayer with JPY currency normalization</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Quotes in JPY, historical volatility, DCF valuation, portfolio covariance estimation</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>7203.T (Toyota), 6758.T (Sony), 9984.T (SoftBank), 6861.T (Keyence), 8035.T (Tokyo Electron)</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>CLI: python run_research.py 7203.T 1
+Quant: cuOpt QP optimization across .T assets</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Australian Equities</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Australian Securities Exchange (ASX, Australia)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Ticker with .AX suffix: &lt;SYMBOL&gt;.AX</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Multi-source DataLayer with AUD currency normalization</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Quotes in AUD, mining/banking fundamentals, DCF valuation, dividend yield tracking</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>BHP.AX (BHP Group), CBA.AX (Commonwealth Bank), CSL.AX (CSL Limited), FMG.AX (Fortescue)</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>CLI: python run_research.py BHP.AX 1
+Watchlist: Add to watchlist.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Exchange Traded Funds (ETFs) &amp; Benchmarks</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Global ETF Markets (US, Global)</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Bare symbol: SPY, QQQ, SMH, etc.</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>BacktestSandbox + AlertMonitor + yFinance Historical Engine</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Benchmark comparative returns, Alpha calculation, Sharpe ratio, Max Drawdown, cuOpt QP optimal weighting</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>SPY (S&amp;P 500), QQQ (Nasdaq 100), SMH (Semiconductors), XLK (Tech), IWM (Russell 2000), VTI (Total US), GLD (Gold)</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>CLI: python -m tools.backtest
+API: sandbox.run_optimized_portfolio_backtest(['AAPL', 'NVDA'], benchmark='QQQ')</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(multi-asset): Part 1 Groundwork - Live Multi-Asset Data Engine, Options/Futures/Commodities/Crypto/Bonds feeds, and Agent Roster
</commit_message>
<xml_diff>
--- a/agents_and_skills_catalog.xlsx
+++ b/agents_and_skills_catalog.xlsx
@@ -530,7 +530,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -574,11 +574,11 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Fundamental, adversarial, audit, and reporting agents</t>
+          <t>Fundamental, derivatives, macro, risk, audit, and reporting agents</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>100% (89/89 Passing)</t>
+          <t>100% Passing</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -670,12 +670,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
@@ -1292,6 +1292,288 @@
       <c r="I13" s="6" t="inlineStr">
         <is>
           <t>Logs execution to ProvenanceLedger with source_tag='R_STUDIO_ECONOMETRICS'</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Meridian Multi-Asset Master Orchestrator</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>MeridianMultiAssetOrchestrator (agents/meridian_orchestrator.py)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Multi-Asset Orchestration</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Coordinates 5 specialized desks (Options, Futures, Macro, Crypto, Risk), aggregates cross-asset portfolios, enforces risk gatekeeping</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Triggered via MeridianMultiAssetOrchestrator.run_multi_asset_committee() or Dashboard Web Terminal</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>agents.meridian_orchestrator.MeridianMultiAssetOrchestrator()</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Multi-asset allocations, desk specs, capital budget</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Institutional Multi-Asset Investment Dossier &amp; Risk Gatekeeper Decision</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>Registers full orchestration run to ProvenanceLedger</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Options Greek Strategist</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>OptionsGreekStrategist (agents/options_greek_agent.py)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Derivatives &amp; Volatility</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Computes Black-Scholes 1st/2nd-order Greeks, implied volatility smiles/skews, multi-leg strategy payoffs, and delta-hedging overlays</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Triggered on options contract queries, strategy backtests, or multi-asset orchestration</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>agents.options_greek_agent.OptionsGreekStrategist()</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Spot price, strike, expiry, volatility, risk-free rate, legs</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Options Greek Sensitivity Matrix &amp; PnL Payoff Distributions</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Logs analytical Greeks and pricing to ProvenanceLedger</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Futures &amp; Commodity Desk Agent</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>FuturesCommodityAgent (agents/futures_commodity_agent.py)</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Commodities &amp; Futures</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Models cost-of-carry pricing, analyzes Contango vs. Backwardation term structures, computes roll yield carry, and stress-tests exchange margins</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Triggered on commodity/futures evaluation or portfolio hedge structuring</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>agents.futures_commodity_agent.FuturesCommodityAgent()</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Futures curve, spot price, storage cost, convenience yield, margin specs</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Term Structure Analysis, Annualized Roll Yield, Margin Call Buffer</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Registers curve metrics &amp; leverage checks to ProvenanceLedger</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Fixed Income Macro Agent</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>FixedIncomeMacroAgent (agents/fixed_income_macro_agent.py)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Rates &amp; Macro</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Analyzes sovereign yield curves (3M to 30Y), detects 2Y-10Y inversions, computes Macaulay/Modified duration, Convexity, and DV01</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Triggered on macro rate reviews, bond portfolio duration checks, or rate shock stress tests</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>agents.fixed_income_macro_agent.FixedIncomeMacroAgent()</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Bond cash flows, coupon rate, YTM, Treasury curve points</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Bond Sensitivity Profile, DV01 per Million Par, Yield Curve Regime Report</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>Logs duration and inversion metrics to ProvenanceLedger</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Crypto &amp; 24/7 Derivatives Agent</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>CryptoDerivativesAgent (agents/crypto_derivatives_agent.py)</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>24/7 Digital Derivatives</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Monitors perpetual swap 8h funding rates, compound APY, cash-and-carry basis arbitrage, and exchange liquidation cascade risks</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Triggered on digital asset derivative surveillance or funding yield capture</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>agents.crypto_derivatives_agent.CryptoDerivativesAgent()</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Perp mark/spot prices, 8h funding rate, open interest, volume, leverage</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>Perpetual Funding APY, Basis Arbitrage Viability, Liquidation Buffer</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>Records funding rates and liquidation distance to ProvenanceLedger</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Cross-Asset Risk Officer</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>CrossAssetRiskOfficer (agents/cross_asset_risk_officer.py)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Risk Oversight &amp; Gatekeeper</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Chief Risk Officer gatekeeper computing Parametric VaR (95%/99%), Expected Shortfall (CVaR), historical crisis stress tests, and Master Red Flags</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Triggered automatically at the conclusion of multi-asset reviews or standalone portfolio risk audits</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>agents.cross_asset_risk_officer.CrossAssetRiskOfficer()</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Cross-asset allocations, volatility vector, correlation matrix, desk reports</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Authoritative Risk Verdict (APPROVED / REJECTED) &amp; Master Red Flags Register</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Tamper-evident audit signature in ProvenanceLedger</t>
         </is>
       </c>
     </row>

</xml_diff>